<commit_message>
feat: enhance booking flow and notification system
- Add dual-channel WhatsApp/SMS notification support
- Expand booking flow with branch and service selection
- Update type definitions for clinical operations
- Integrate Firebase, PDF generation, and confetti
- Improve PWA configuration and cache settings
</commit_message>
<xml_diff>
--- a/data/patients_records.xlsx
+++ b/data/patients_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:AB3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -424,72 +424,265 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Booking Ref</v>
+        <v>bookingRef</v>
       </c>
       <c r="B1" t="str">
-        <v>Booking Date</v>
+        <v>bookingDate</v>
       </c>
       <c r="C1" t="str">
-        <v>Patient Name</v>
+        <v>patientName</v>
       </c>
       <c r="D1" t="str">
-        <v>First Name</v>
+        <v>firstName</v>
       </c>
       <c r="E1" t="str">
-        <v>Last Name</v>
+        <v>lastName</v>
       </c>
       <c r="F1" t="str">
-        <v>Phone</v>
+        <v>phone</v>
       </c>
       <c r="G1" t="str">
-        <v>Email</v>
+        <v>email</v>
       </c>
       <c r="H1" t="str">
-        <v>Date of Birth</v>
+        <v>dob</v>
       </c>
       <c r="I1" t="str">
-        <v>Patient Type</v>
+        <v>patientType</v>
       </c>
       <c r="J1" t="str">
-        <v>Branch Name</v>
+        <v>branchName</v>
       </c>
       <c r="K1" t="str">
-        <v>Branch Address</v>
+        <v>branchAddress</v>
       </c>
       <c r="L1" t="str">
-        <v>Branch Phone</v>
+        <v>branchPhone</v>
       </c>
       <c r="M1" t="str">
-        <v>Treatment Name</v>
+        <v>branchId</v>
       </c>
       <c r="N1" t="str">
-        <v>Duration</v>
+        <v>treatmentName</v>
       </c>
       <c r="O1" t="str">
-        <v>Estimated Fee</v>
+        <v>treatmentDuration</v>
       </c>
       <c r="P1" t="str">
-        <v>Dentist Name</v>
+        <v>estimatedFee</v>
       </c>
       <c r="Q1" t="str">
-        <v>Specialization</v>
+        <v>doctorName</v>
       </c>
       <c r="R1" t="str">
-        <v>Appointment Date</v>
+        <v>doctorSpecialization</v>
       </c>
       <c r="S1" t="str">
-        <v>Appointment Time</v>
+        <v>appointmentDate</v>
       </c>
       <c r="T1" t="str">
-        <v>Notes</v>
+        <v>appointmentTime</v>
       </c>
       <c r="U1" t="str">
-        <v>Status</v>
+        <v>notes</v>
+      </c>
+      <c r="V1" t="str">
+        <v>status</v>
+      </c>
+      <c r="W1" t="str">
+        <v>paymentMode</v>
+      </c>
+      <c r="X1" t="str">
+        <v>paymentStatus</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>paymentRef</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>amountPaidNow</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>amountRemaining</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>attachmentName</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SCWN2MG</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-09-18 10:24</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Karan Kshirsagar</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Kshirsagar</v>
+      </c>
+      <c r="F2" t="str">
+        <v>9527050086</v>
+      </c>
+      <c r="G2" t="str">
+        <v>karanrk2005@gmail.com</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Not specified</v>
+      </c>
+      <c r="I2" t="str">
+        <v>New patient</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Smart Dental Clinic – Downtown Central (Main)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>102 Wellness Plaza, Dental Street, Medical Hub, Central City - 400001</v>
+      </c>
+      <c r="L2" t="str">
+        <v>+91 98765 00000</v>
+      </c>
+      <c r="M2" t="str">
+        <v>branch-1</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Composite Tooth-Colored Filling</v>
+      </c>
+      <c r="O2" t="str">
+        <v>35 min</v>
+      </c>
+      <c r="P2" t="str">
+        <v>₹1,000 – ₹2,200</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Dr. Vikram Shah</v>
+      </c>
+      <c r="R2" t="str">
+        <v>General Dental Surgeon</v>
+      </c>
+      <c r="S2" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="T2" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="U2" t="str">
+        <v>None</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Pay at Clinic Counter</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Pending at Clinic Counter</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>₹0</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>₹1,000 – ₹2,200</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>None</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SCXOCCJ</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-09-18 09:55</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Karan Kshirsagar</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Kshirsagar</v>
+      </c>
+      <c r="F3" t="str">
+        <v>9527050086</v>
+      </c>
+      <c r="G3" t="str">
+        <v>karanrk2005@gmail.com</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Not specified</v>
+      </c>
+      <c r="I3" t="str">
+        <v>New patient</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Smart Dental Clinic – Downtown Central (Main)</v>
+      </c>
+      <c r="K3" t="str">
+        <v>102 Wellness Plaza, Dental Street, Medical Hub, Central City - 400001</v>
+      </c>
+      <c r="L3" t="str">
+        <v>+91 98765 00000</v>
+      </c>
+      <c r="M3" t="str">
+        <v>branch-1</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Tooth Sensitivity Relief</v>
+      </c>
+      <c r="O3" t="str">
+        <v>30 min</v>
+      </c>
+      <c r="P3" t="str">
+        <v>₹600 – ₹1,500</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Dr. Vikram Shah</v>
+      </c>
+      <c r="R3" t="str">
+        <v>General Dental Surgeon</v>
+      </c>
+      <c r="S3" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="T3" t="str">
+        <v>10:00 AM</v>
+      </c>
+      <c r="U3" t="str">
+        <v>None</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Advance Paid (₹600)</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Advance Paid (₹600) · Remaining ₹0</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>₹600</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>₹0</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>None</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement real-time admin sync for booking data
Add event listeners to update doctors, treatments, and clinic timings dynamically when admin changes occur. Sync active bookings with updated catalog data to ensure validity, and refine treatment filtering logic for branch-specific services.
</commit_message>
<xml_diff>
--- a/data/patients_records.xlsx
+++ b/data/patients_records.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Patient Records" sheetId="1" r:id="rId1"/>
+    <sheet name="Records (September 2026)" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AC5"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -507,13 +507,16 @@
       <c r="AB1" t="str">
         <v>attachmentName</v>
       </c>
+      <c r="AC1" t="str">
+        <v>reminder2hSent</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SCWN2MG</v>
+        <v>SCMX2V4</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-18 10:24</v>
+        <v>2026-09-28 07:38</v>
       </c>
       <c r="C2" t="str">
         <v>Karan Kshirsagar</v>
@@ -549,13 +552,13 @@
         <v>branch-1</v>
       </c>
       <c r="N2" t="str">
-        <v>Composite Tooth-Colored Filling</v>
+        <v>Dental X-Ray (OPG &amp; Bitewing)</v>
       </c>
       <c r="O2" t="str">
-        <v>35 min</v>
+        <v>15 min</v>
       </c>
       <c r="P2" t="str">
-        <v>₹1,000 – ₹2,200</v>
+        <v>₹600 – ₹1,000</v>
       </c>
       <c r="Q2" t="str">
         <v>Dr. Vikram Shah</v>
@@ -564,31 +567,31 @@
         <v>General Dental Surgeon</v>
       </c>
       <c r="S2" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-30</v>
       </c>
       <c r="T2" t="str">
-        <v>10:30 AM</v>
+        <v>5:30 PM</v>
       </c>
       <c r="U2" t="str">
-        <v>None</v>
+        <v>Updated from admin edit modal test</v>
       </c>
       <c r="V2" t="str">
         <v>Confirmed</v>
       </c>
       <c r="W2" t="str">
-        <v>Pay at Clinic Counter</v>
+        <v>Advance Paid (₹600)</v>
       </c>
       <c r="X2" t="str">
-        <v>Pending at Clinic Counter</v>
+        <v>Advance Paid (₹600) · Remaining ₹0</v>
       </c>
       <c r="Y2" t="str">
         <v>N/A</v>
       </c>
       <c r="Z2" t="str">
+        <v>₹600</v>
+      </c>
+      <c r="AA2" t="str">
         <v>₹0</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>₹1,000 – ₹2,200</v>
       </c>
       <c r="AB2" t="str">
         <v>None</v>
@@ -596,22 +599,22 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SCXOCCJ</v>
+        <v>SCJXXRQ</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-18 09:55</v>
+        <v>2026-09-28 07:38</v>
       </c>
       <c r="C3" t="str">
-        <v>Karan Kshirsagar</v>
+        <v>piu  kadam</v>
       </c>
       <c r="D3" t="str">
-        <v>Karan</v>
+        <v>piu</v>
       </c>
       <c r="E3" t="str">
-        <v>Kshirsagar</v>
+        <v xml:space="preserve"> kadam</v>
       </c>
       <c r="F3" t="str">
-        <v>9527050086</v>
+        <v>12345674</v>
       </c>
       <c r="G3" t="str">
         <v>karanrk2005@gmail.com</v>
@@ -635,22 +638,22 @@
         <v>branch-1</v>
       </c>
       <c r="N3" t="str">
-        <v>Tooth Sensitivity Relief</v>
+        <v>Consultation &amp; Checkup</v>
       </c>
       <c r="O3" t="str">
         <v>30 min</v>
       </c>
       <c r="P3" t="str">
-        <v>₹600 – ₹1,500</v>
+        <v>₹300 – ₹800</v>
       </c>
       <c r="Q3" t="str">
-        <v>Dr. Vikram Shah</v>
+        <v>Dr. Priya Mehta</v>
       </c>
       <c r="R3" t="str">
-        <v>General Dental Surgeon</v>
+        <v>General &amp; Preventive Dentistry</v>
       </c>
       <c r="S3" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-28</v>
       </c>
       <c r="T3" t="str">
         <v>10:00 AM</v>
@@ -662,27 +665,202 @@
         <v>Confirmed</v>
       </c>
       <c r="W3" t="str">
-        <v>Advance Paid (₹600)</v>
+        <v>Advance Paid (₹300)</v>
       </c>
       <c r="X3" t="str">
-        <v>Advance Paid (₹600) · Remaining ₹0</v>
+        <v>Advance Paid (₹300) · Remaining ₹0</v>
       </c>
       <c r="Y3" t="str">
         <v>N/A</v>
       </c>
       <c r="Z3" t="str">
-        <v>₹600</v>
+        <v>₹300</v>
       </c>
       <c r="AA3" t="str">
         <v>₹0</v>
       </c>
       <c r="AB3" t="str">
+        <v>None</v>
+      </c>
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SCWN2MG</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-09-18 10:24</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Karan Kshirsagar</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Kshirsagar</v>
+      </c>
+      <c r="F4" t="str">
+        <v>9527050086</v>
+      </c>
+      <c r="G4" t="str">
+        <v>karanrk2005@gmail.com</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Not specified</v>
+      </c>
+      <c r="I4" t="str">
+        <v>New patient</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Smart Dental Clinic – Downtown Central (Main)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>102 Wellness Plaza, Dental Street, Medical Hub, Central City - 400001</v>
+      </c>
+      <c r="L4" t="str">
+        <v>+91 98765 00000</v>
+      </c>
+      <c r="M4" t="str">
+        <v>branch-1</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Composite Tooth-Colored Filling</v>
+      </c>
+      <c r="O4" t="str">
+        <v>35 min</v>
+      </c>
+      <c r="P4" t="str">
+        <v>₹1,000 – ₹2,200</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Dr. Vikram Shah</v>
+      </c>
+      <c r="R4" t="str">
+        <v>General Dental Surgeon</v>
+      </c>
+      <c r="S4" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="T4" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="U4" t="str">
+        <v>None</v>
+      </c>
+      <c r="V4" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="W4" t="str">
+        <v>Pay at Clinic Counter</v>
+      </c>
+      <c r="X4" t="str">
+        <v>Pending at Clinic Counter</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>₹0</v>
+      </c>
+      <c r="AA4" t="str">
+        <v>₹1,000 – ₹2,200</v>
+      </c>
+      <c r="AB4" t="str">
+        <v>None</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SCXOCCJ</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-09-18 09:55</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Karan Kshirsagar</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Kshirsagar</v>
+      </c>
+      <c r="F5" t="str">
+        <v>9527050086</v>
+      </c>
+      <c r="G5" t="str">
+        <v>karanrk2005@gmail.com</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Not specified</v>
+      </c>
+      <c r="I5" t="str">
+        <v>New patient</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Smart Dental Clinic – Downtown Central (Main)</v>
+      </c>
+      <c r="K5" t="str">
+        <v>102 Wellness Plaza, Dental Street, Medical Hub, Central City - 400001</v>
+      </c>
+      <c r="L5" t="str">
+        <v>+91 98765 00000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>branch-1</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Tooth Sensitivity Relief</v>
+      </c>
+      <c r="O5" t="str">
+        <v>30 min</v>
+      </c>
+      <c r="P5" t="str">
+        <v>₹600 – ₹1,500</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Dr. Vikram Shah</v>
+      </c>
+      <c r="R5" t="str">
+        <v>General Dental Surgeon</v>
+      </c>
+      <c r="S5" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="T5" t="str">
+        <v>10:00 AM</v>
+      </c>
+      <c r="U5" t="str">
+        <v>None</v>
+      </c>
+      <c r="V5" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="W5" t="str">
+        <v>Advance Paid (₹600)</v>
+      </c>
+      <c r="X5" t="str">
+        <v>Advance Paid (₹600) · Remaining ₹0</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>₹600</v>
+      </c>
+      <c r="AA5" t="str">
+        <v>₹0</v>
+      </c>
+      <c r="AB5" t="str">
         <v>None</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>